<commit_message>
auto: timetable update from Sadashiv Bhimanna <sadashiv.bhimanna@nmims.edu>
</commit_message>
<xml_diff>
--- a/downloads/10.08.2026 to 16.08.2026-2nd.xlsx
+++ b/downloads/10.08.2026 to 16.08.2026-2nd.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sadashiv.bhimanna\Desktop\2026-27\Second Year Time Table\Weekly time table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672F9EF8-C4A3-4BA5-897E-3073DD08F114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F1D088-8A6A-46FB-927A-CD209481D032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
   <si>
     <t>Day/
 Time</t>
@@ -235,12 +235,6 @@
     <t>R&amp; S
 Hybrid
 (6:30 pm to 8:00pm)</t>
-  </si>
-  <si>
-    <t>BS Div A
-Rescheduled class
-L06, 2nd floor
-Dr Srividya Raghavan</t>
   </si>
   <si>
     <t>CB
@@ -868,7 +862,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1073,9 +1067,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1144,6 +1135,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1443,18 +1440,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="87" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
+      <c r="A1" s="86" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="87"/>
+      <c r="J1" s="87"/>
     </row>
     <row r="2" spans="1:10" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1475,10 +1472,10 @@
       <c r="F2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="91" t="s">
+      <c r="G2" s="90" t="s">
         <v>38</v>
       </c>
-      <c r="H2" s="92"/>
+      <c r="H2" s="91"/>
       <c r="I2" s="45" t="s">
         <v>36</v>
       </c>
@@ -1487,7 +1484,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="93" t="s">
+      <c r="A3" s="92" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="61"/>
@@ -1497,7 +1494,7 @@
       <c r="D3" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="94" t="s">
+      <c r="E3" s="93" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="7" t="s">
@@ -1513,11 +1510,11 @@
       <c r="J3" s="56"/>
     </row>
     <row r="4" spans="1:10" ht="65.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="90"/>
-      <c r="B4" s="76"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="95"/>
+      <c r="A4" s="89"/>
+      <c r="B4" s="75"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="94"/>
       <c r="F4" s="11" t="s">
         <v>12</v>
       </c>
@@ -1529,7 +1526,7 @@
       <c r="J4" s="53"/>
     </row>
     <row r="5" spans="1:10" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="90" t="s">
+      <c r="A5" s="89" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="42" t="s">
@@ -1541,7 +1538,7 @@
       <c r="D5" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="95"/>
+      <c r="E5" s="94"/>
       <c r="F5" s="66" t="s">
         <v>12</v>
       </c>
@@ -1553,11 +1550,11 @@
       <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:10" ht="65.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="90"/>
+      <c r="A6" s="89"/>
       <c r="B6" s="14"/>
       <c r="C6" s="15"/>
       <c r="D6" s="16"/>
-      <c r="E6" s="95"/>
+      <c r="E6" s="94"/>
       <c r="F6" s="31" t="s">
         <v>21</v>
       </c>
@@ -1569,7 +1566,7 @@
       <c r="J6" s="53"/>
     </row>
     <row r="7" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="90" t="s">
+      <c r="A7" s="89" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="18"/>
@@ -1579,7 +1576,7 @@
       <c r="D7" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="95"/>
+      <c r="E7" s="94"/>
       <c r="F7" s="20" t="s">
         <v>26</v>
       </c>
@@ -1593,7 +1590,7 @@
       <c r="J7" s="53"/>
     </row>
     <row r="8" spans="1:10" ht="63.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="90"/>
+      <c r="A8" s="89"/>
       <c r="B8" s="14"/>
       <c r="C8" s="9" t="s">
         <v>23</v>
@@ -1601,7 +1598,7 @@
       <c r="D8" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="95"/>
+      <c r="E8" s="94"/>
       <c r="F8" s="23"/>
       <c r="G8" s="24" t="s">
         <v>18</v>
@@ -1611,7 +1608,7 @@
       <c r="J8" s="55"/>
     </row>
     <row r="9" spans="1:10" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="90" t="s">
+      <c r="A9" s="89" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="25" t="s">
@@ -1623,7 +1620,7 @@
       <c r="D9" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="95"/>
+      <c r="E9" s="94"/>
       <c r="F9" s="27" t="s">
         <v>26</v>
       </c>
@@ -1639,13 +1636,13 @@
       <c r="J9" s="57"/>
     </row>
     <row r="10" spans="1:10" ht="69" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="90"/>
+      <c r="A10" s="89"/>
       <c r="B10" s="29"/>
       <c r="C10" s="31"/>
       <c r="D10" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="95"/>
+      <c r="E10" s="94"/>
       <c r="F10" s="43"/>
       <c r="G10" s="31" t="s">
         <v>39</v>
@@ -1654,23 +1651,23 @@
         <v>40</v>
       </c>
       <c r="I10" s="28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J10" s="70"/>
     </row>
     <row r="11" spans="1:10" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="89" t="s">
+      <c r="A11" s="88" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="84"/>
-      <c r="C11" s="79" t="s">
+      <c r="B11" s="83"/>
+      <c r="C11" s="78" t="s">
         <v>30</v>
       </c>
       <c r="D11" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="95"/>
-      <c r="F11" s="64" t="s">
+      <c r="E11" s="94"/>
+      <c r="F11" s="95" t="s">
         <v>42</v>
       </c>
       <c r="G11" s="41" t="s">
@@ -1678,12 +1675,12 @@
       </c>
       <c r="H11" s="44"/>
       <c r="I11" s="59" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J11" s="56"/>
     </row>
     <row r="12" spans="1:10" ht="63.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="90"/>
+      <c r="A12" s="89"/>
       <c r="B12" s="71"/>
       <c r="C12" s="31" t="s">
         <v>31</v>
@@ -1691,19 +1688,19 @@
       <c r="D12" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="95"/>
-      <c r="F12" s="72"/>
-      <c r="G12" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="H12" s="73"/>
+      <c r="E12" s="94"/>
+      <c r="F12" s="96"/>
+      <c r="G12" s="76" t="s">
+        <v>42</v>
+      </c>
+      <c r="H12" s="72"/>
       <c r="I12" s="6" t="s">
         <v>15</v>
       </c>
       <c r="J12" s="53"/>
     </row>
     <row r="13" spans="1:10" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="89" t="s">
+      <c r="A13" s="88" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="52"/>
@@ -1714,26 +1711,26 @@
         <v>34</v>
       </c>
       <c r="E13" s="35"/>
-      <c r="F13" s="82" t="s">
+      <c r="F13" s="81" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="83" t="s">
+      <c r="G13" s="82" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="78"/>
-      <c r="I13" s="80"/>
+      <c r="H13" s="77"/>
+      <c r="I13" s="79"/>
       <c r="J13" s="53"/>
     </row>
     <row r="14" spans="1:10" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="90"/>
+      <c r="A14" s="89"/>
       <c r="B14" s="36"/>
-      <c r="C14" s="85"/>
-      <c r="D14" s="86"/>
+      <c r="C14" s="84"/>
+      <c r="D14" s="85"/>
       <c r="E14" s="37"/>
       <c r="F14" s="23"/>
       <c r="G14" s="38"/>
       <c r="H14" s="33"/>
-      <c r="I14" s="81"/>
+      <c r="I14" s="80"/>
       <c r="J14" s="54"/>
     </row>
   </sheetData>

</xml_diff>